<commit_message>
update conversational web view
</commit_message>
<xml_diff>
--- a/samples/NVDA_analysis.xlsx
+++ b/samples/NVDA_analysis.xlsx
@@ -7311,7 +7311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7354,111 +7354,999 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2022-11-30</t>
+          <t>2022-11-16</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Product Launch</t>
+          <t>Partnership</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>OpenAI launches ChatGPT, igniting generative-AI demand cycle</t>
+          <t>Nvidia and Microsoft partner to build massive AI cloud supercomputer</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>ChatGPT's launch kicked off the generative-AI demand cycle, driving massive demand for NVIDIA's data-center GPUs used to train and run large language models.</t>
+          <t>Nvidia and Microsoft announced a multi-year collaboration to build a large-scale cloud AI supercomputer on Azure using tens of thousands of Nvidia GPUs, expanding Nvidia's data-center footprint via a major hyperscaler.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://openai.com/blog/chatgpt</t>
+          <t>https://arstechnica.com/information-technology/2022/11/nvidia-and-microsoft-team-up-to-build-massive-ai-cloud-computer/, https://www.reuters.com/technology/nvidia-says-it-is-working-with-microsoft-build-massive-cloud-ai-computer-2022-11-16/, https://www.hpcwire.com/off-the-wire/nvidia-teams-with-microsoft-to-build-massive-cloud-ai-computer/, https://www.theverge.com/2022/11/17/23464001/nvidia-microsoft-ai-supercomputer-announcement</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://openai.com/blog/chatgpt</t>
+          <t>https://arstechnica.com/information-technology/2022/11/nvidia-and-microsoft-team-up-to-build-massive-ai-cloud-computer/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2023-03-14</t>
+          <t>2022-11-09</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Product Launch</t>
+          <t>Regulatory</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>OpenAI releases GPT-4 with multimodal capabilities</t>
+          <t>Nvidia introduces A800 GPU to circumvent U.S. China export restrictions</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>GPT-4's launch intensified enterprise AI compute demand, a tailwind for NVIDIA's GPU sales as adoption of larger models scales training and inference needs.</t>
+          <t>Nvidia created a slowed-down A800 chip for the Chinese market to comply with new U.S. export controls, highlighting regulatory risk to a significant revenue market.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://openai.com/research/gpt-4</t>
+          <t>https://www.theverge.com/2022/11/8/23447886/nvidia-a800-china-chip-ai-research-slowed-down-restrictions</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://openai.com/research/gpt-4</t>
+          <t>https://www.theverge.com/2022/11/8/23447886/nvidia-a800-china-chip-ai-research-slowed-down-restrictions</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2022-11-14</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Nvidia bundles enterprise AI software with H100 systems at SC22</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Nvidia announced broad H100 and Quantum-2 adoption and bundled enterprise AI software with new H100 systems, strengthening its flagship data-center product ramp.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.theregister.com/2022/11/14/nvidia_h100_software_bundle/, https://wandb.ai/telidavies/ml-news/reports/NVIDIA-SC22-Widespread-H100-Quantum-2-Adoption-Omniverse-Library-Updates--VmlldzoyOTY5NzQw</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://www.theregister.com/2022/11/14/nvidia_h100_software_bundle/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2022-12-01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Supply Chain</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TSMC to make 4nm chips in Arizona for Apple, AMD and Nvidia</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TSMC's Arizona 4nm fab plans include Nvidia, relevant to supply chain diversification and geopolitical resilience for Nvidia's advanced chip production.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://techmonitor.ai/technology/silicon/tsmcs-arizona-apple-amd-nvidia</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://techmonitor.ai/technology/silicon/tsmcs-arizona-apple-amd-nvidia</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2023-02-23</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Earnings</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Nvidia fiscal Q4 earnings show growing lead in AI chip race</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Nvidia's earnings and bullish AI commentary drove a ~12% stock move and demonstrated its expanding data-center/AI momentum amid the generative AI boom.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/technology/nvidia-results-show-its-growing-lead-ai-chip-race-2023-02-23/, https://www.cnbc.com/2023/02/23/nvidia-stock-up-12percent-on-earnings-ai-potential.html, https://venturebeat.com/ai/how-nvidia-dominated-ai-and-plans-to-keep-it-that-way-as-generative-ai-explodes/, https://www.cnbc.com/2023/02/23/nvidias-a100-is-the-10000-chip-powering-the-race-for-ai-.html</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/technology/nvidia-results-show-its-growing-lead-ai-chip-race-2023-02-23/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2023-02-13</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Management Commentary</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Nvidia CEO calls ChatGPT the 'iPhone moment of AI'</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Jensen Huang framing ChatGPT as AI's iPhone moment signals strategic positioning around generative AI demand, widely echoed in coverage.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://wccftech.com/nvidia-ceo-calls-chatgpt-as-one-of-the-greatest-thing-ever-done-for-computing-says-its-the-iphone-moment-of-ai/</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://wccftech.com/nvidia-ceo-calls-chatgpt-as-one-of-the-greatest-thing-ever-done-for-computing-says-its-the-iphone-moment-of-ai/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2023-03-21</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Nvidia GTC 2023: DGX Cloud, inference platforms, and cloud partnerships</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>At GTC, Nvidia launched DGX Cloud, new inference platforms for LLMs/generative AI, and partnerships to bring next-gen AI chips to AWS and Google Cloud, broadly expanding its generative-AI product strategy.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://nvidianews.nvidia.com/news/nvidia-launches-inference-platforms-for-large-language-models-and-generative-ai-workloads, https://nvidianews.nvidia.com/news/nvidia-launches-dgx-cloud-giving-every-enterprise-instant-access-to-ai-supercomputer-from-a-browser, https://techcrunch.com/2023/03/21/nvidia-partners-with-google-cloud-to-launch-ai-focused-hardware-instances/, https://www.bloomberg.com/news/articles/2023-03-21/nvidia-s-next-gen-ai-chips-are-coming-to-aws-and-google-cloud, https://www.zdnet.com/article/for-ais-iphone-moment-in-chatgpt-nvidia-unveils-a-large-language-model-chip/, https://blogs.nvidia.com/blog/2023/03/21/gtc-keynote-spring-2023/, https://www.engadget.com/nvidia-gtc-ai-dgx-cloud-161517378.html</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://nvidianews.nvidia.com/news/nvidia-launches-inference-platforms-for-large-language-models-and-generative-ai-workloads</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2023-03-22</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Nvidia and Microsoft to bring industrial metaverse and AI to Azure enterprise users</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Extension of the Microsoft partnership to deliver Omniverse-based industrial metaverse and AI via Azure to enterprise users.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://nvidianews.nvidia.com/news/nvidia-and-microsoft-to-bring-the-industrial-metaverse-and-ai-to-hundreds-of-millions-of-enterprise-users-via-azure-cloud</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://nvidianews.nvidia.com/news/nvidia-and-microsoft-to-bring-the-industrial-metaverse-and-ai-to-hundreds-of-millions-of-enterprise-users-via-azure-cloud</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2023-03-27</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Nvidia H100 NVL for high-end LLM inference launched</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Nvidia launched the H100 NVL variant targeting large language model inference, extending its data-center product portfolio for generative AI workloads.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://www.servethehome.com/nvidia-h100-nvl-for-high-end-ai-inference-launched/</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://www.servethehome.com/nvidia-h100-nvl-for-high-end-ai-inference-launched/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2023-04-05</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Google claims its TPU AI supercomputer beats Nvidia A100</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Google published claims that its TPU v4 supercomputer is faster and greener than Nvidia's A100, signaling competitive pressure from hyperscaler custom silicon.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/technology/google-says-its-ai-supercomputer-is-faster-greener-than-nvidia-2023-04-05/, https://www.cnbc.com/2023/04/05/google-reveals-its-newest-ai-supercomputer-claims-it-beats-nvidia-.html, https://www.msn.com/en-us/money/other/google-says-its-ai-supercomputer-is-faster-greener-than-nvidia-a100-chip/ar-AA19u62B</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/technology/google-says-its-ai-supercomputer-is-faster-greener-than-nvidia-2023-04-05/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2023-04-18</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Microsoft reportedly developing its own AI chips (Athena)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Reports that Microsoft is building its own AI chip and teaming with AMD could reduce future dependence on Nvidia GPUs from a key hyperscaler customer.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://www.theverge.com/2023/4/18/23687912/microsoft-athena-ai-chips-nvidia, https://arstechnica.com/gadgets/2023/05/microsoft-and-amd-are-allegedly-teaming-up-to-combat-nvidias-ai-dominance/, https://www.theverge.com/2023/5/5/23712242/microsoft-amd-ai-processor-chip-nvidia-gpu-athena-mi300</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://www.theverge.com/2023/4/18/23687912/microsoft-athena-ai-chips-nvidia</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2023-04-14</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Nvidia H100 chips selling for over $40k on eBay amid shortage</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Secondary-market H100 prices exceeding $40k and reports of 40% price increases and shortages through December underscore intense demand and pricing power for Nvidia AI GPUs.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://www.cnbc.com/2023/04/14/nvidias-h100-ai-chips-selling-for-more-than-40000-on-ebay.html, https://wccftech.com/nvidia-ai-gpu-demand-blows-up-chip-prices-increase-40-percent-stock-shortages-till-december/</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://www.cnbc.com/2023/04/14/nvidias-h100-ai-chips-selling-for-more-than-40000-on-ebay.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2023-04-25</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Nvidia releases NeMo Guardrails open-source software for AI chatbots</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Nvidia released open-source guardrails software to add safety controls to AI chatbots, expanding its AI software stack.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>https://blogs.nvidia.com/blog/2023/04/25/ai-chatbot-guardrails-nemo/</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://blogs.nvidia.com/blog/2023/04/25/ai-chatbot-guardrails-nemo/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>2023-05-24</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Dell and Nvidia introduce Project Helix for on-premises generative AI</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Dell-Nvidia Project Helix targets secure on-premises generative AI deployments, broadening Nvidia's enterprise generative-AI go-to-market.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>https://nvidianews.nvidia.com/news/dell-technologies-and-nvidia-introduce-project-helix-for-secure-on-premises-generative-ai</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>https://nvidianews.nvidia.com/news/dell-technologies-and-nvidia-introduce-project-helix-for-secure-on-premises-generative-ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2023-05-24</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>Earnings</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>NVIDIA reports blowout Q1 FY24 data-center revenue and guidance</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>NVIDIA guided revenue far above expectations on AI data-center demand and the stock gapped up, directly validating the AI-driven growth thesis for the company.</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://nvidianews.nvidia.com/news/nvidia-announces-financial-results-for-first-quarter-fiscal-2024</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>https://nvidianews.nvidia.com/news/nvidia-announces-financial-results-for-first-quarter-fiscal-2024</t>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Nvidia fiscal Q1 earnings blowout forecast ignites $200B+ AI rally</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Nvidia's blowout revenue guidance driven by AI demand triggered a massive stock surge and hundreds of billions in market-cap gains, a pivotal financial event.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>https://www.wsj.com/articles/nvidia-nvda-q1-earnings-report-2024-132e3559, https://www.reuters.com/technology/nvidia-forecasts-second-quarter-revenue-above-estimates-2023-05-24/, https://www.cnn.com/2023/05/25/tech/nvidia-earnings-ai/index.html, https://www.bloomberg.com/news/articles/2023-05-24/nvidia-ignites-ai-related-stock-rally-after-blow-out-forecast, https://www.marketwatch.com/story/nvidia-barrels-toward-rare-1-trillion-valuation-after-putting-a-dollar-figure-on-ai-boost-443b7d0f</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>https://www.wsj.com/articles/nvidia-nvda-q1-earnings-report-2024-132e3559</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2023-05-29</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Nvidia announces DGX GH200 supercomputer, Grace Hopper in full production, and Ace for Games</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>At Computex, Nvidia unveiled the DGX GH200 AI supercomputer, MGX systems, Grace Hopper superchips in full production, SoftBank/WPP partnerships and generative-AI NPC tech (ACE), a broad product and partnership expansion.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>https://www.tomshardware.com/news/nvidia-unveils-dgx-gh200-supercomputer-and-mgx-systems-grace-hopper-superchips-in-production, https://nvidianews.nvidia.com/news/nvidia-announces-dgx-gh200-ai-supercomputer, https://www.anandtech.com/show/18877/nvidia-grace-hopper-has-entered-full-production-announcing-dgx-gh200-ai-supercomputer, https://nvidianews.nvidia.com/news/softbank-telecom-data-centers-grace-hopper, https://www.cnn.com/2023/05/29/tech/nvidia-wpp-ai-advertising/index.html, https://developer.nvidia.com/blog/generative-ai-sparks-life-into-virtual-characters-with-ace-for-games/, https://www.bloomberg.com/news/articles/2023-05-29/nvidia-nvda-unveils-more-ai-products-to-further-capitalize-on-frenzy</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>https://www.tomshardware.com/news/nvidia-unveils-dgx-gh200-supercomputer-and-mgx-systems-grace-hopper-superchips-in-production</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2023-05-30</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Nvidia becomes first chipmaker to reach $1 trillion market value</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Nvidia crossed a $1 trillion market capitalization on booming AI demand, a landmark valuation milestone reflecting its AI leadership.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>https://www.theguardian.com/business/2023/may/30/nvidia-chipmaker-value-ai-chip-shares-artificial-intelligence, https://www.reuters.com/technology/nvidia-sets-eye-1-trillion-market-value-2023-05-30/, https://www.theverge.com/2023/5/30/23742123/nvidia-stock-ai-gpu-1-trillion-market-cap-price-value, https://www.wsj.com/articles/nvidia-ai-chips-jensen-huang-dennys-d3226926</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.theguardian.com/business/2023/may/30/nvidia-chipmaker-value-ai-chip-shares-artificial-intelligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2023-06-06</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Nvidia unveils Spectrum-X Ethernet networking for AI</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Nvidia announced a new AI-focused Ethernet platform (Spectrum-X) and Grace Hopper superchip in full production, expanding its networking portfolio amid competitive scrutiny of InfiniBand.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>https://www.zdnet.com/article/nvidia-unveils-new-kind-of-ethernet-for-ai-grace-hopper-superchip-in-full-production/, https://www.nextplatform.com/2023/05/25/nvidia-hints-at-upcoming-ai-focused-spectrum-4-ethernet/, https://www.nvidia.com/en-us/data-center/grace-hopper-superchip/</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.zdnet.com/article/nvidia-unveils-new-kind-of-ethernet-for-ai-grace-hopper-superchip-in-full-production/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2023-06-13</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Competition</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>AMD unveils MI300X GPU to challenge Nvidia's AI dominance</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>AMD launched the MI300X AI GPU and plans to ramp production, representing the most direct competitive threat to Nvidia's data-center AI GPU supremacy.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/technology/amd-likely-offer-details-ai-chip-challenge-nvidia-2023-06-13/, https://www.cnbc.com/2023/06/13/amd-reveals-new-ai-chip-to-challenge-nvidias-dominance.html, https://www.news.upveda.in/2023/06/13/amd-unveils-mi300x-its-advanced-ai-gpu-to-challenge-nvidias-dominance/, https://www.reuters.com/technology/amds-ai-chips-could-match-nvidias-offerings-software-firm-says-2023-06-30/</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/technology/amd-likely-offer-details-ai-chip-challenge-nvidia-2023-06-13/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2023-06-09</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Nvidia NeMo AI software found vulnerable to data-leak exploit</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Researchers tricked Nvidia's AI software into leaking data, raising security concerns about its enterprise AI software offerings.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>https://arstechnica.com/gadgets/2023/06/nvidias-ai-software-tricked-into-leaking-data/, https://www.ft.com/content/5aceb7a6-9d5a-4f1f-af3d-1ef0129b0934</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://arstechnica.com/gadgets/2023/06/nvidias-ai-software-tricked-into-leaking-data/</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2023-06-19</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ByteDance reportedly bought $1B of Nvidia GPUs; China gray market emerges</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Reports of ByteDance spending $1B on Nvidia GPUs and an underground China market for high-end chips highlight strong Chinese demand amid export-control pressures.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>https://www.tomshardware.com/news/chinas-bytedance-has-gobbled-up-dollar1-billion-of-nvidia-gpus-for-ai-this-year, https://www.reuters.com/technology/inside-chinas-underground-market-high-end-nvidia-ai-chips-2023-06-19/</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.tomshardware.com/news/chinas-bytedance-has-gobbled-up-dollar1-billion-of-nvidia-gpus-for-ai-this-year</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2023-06-28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Regulatory</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Report of new U.S. ban on AI chip exports to China hits Nvidia shares</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Reports of a potential new Biden administration ban on AI chip exports to China pressured Nvidia and AMD stocks, signaling material regulatory risk to China revenue.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>https://www.marketwatch.com/story/nvidia-amd-stocks-fall-on-report-of-new-ai-chip-bans-from-biden-administration-a8574751</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.marketwatch.com/story/nvidia-amd-stocks-fall-on-report-of-new-ai-chip-bans-from-biden-administration-a8574751</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2023-06-27</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Nvidia partners with Snowflake for generative AI in the data cloud</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Nvidia brought its AI computing platform to Snowflake to enable generative AI development on enterprise data, expanding enterprise adoption channels.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/technology/nvidia-brings-its-ai-computing-platform-cloud-data-firm-snowflake-2023-06-27/, https://www.snowflake.com/news/snowflake-and-nvidia-team-to-help-businesses-harness-their-data-for-generative-ai-in-the-data-cloud/, https://venturebeat.com/ai/snowflake-nvidia-partner-enable-generative-ai-application-development-snowflake-data-cloud/</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.reuters.com/technology/nvidia-brings-its-ai-computing-platform-cloud-data-firm-snowflake-2023-06-27/</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2023-06-27</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>H100 GPUs set records in debut MLPerf generative AI benchmark</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Nvidia's H100 GPUs set the standard in the first generative AI MLPerf benchmark, reinforcing performance leadership claims.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://blogs.nvidia.com/blog/2023/06/27/generative-ai-debut-mlperf/</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://blogs.nvidia.com/blog/2023/06/27/generative-ai-debut-mlperf/</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2023-06-29</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Investment</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Nvidia backs multiple AI startups: Inflection AI, Cohere, Runway</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Nvidia participated in large funding rounds for Inflection AI ($1.3B, deploying 22,000 H100s), Cohere ($270M), and Runway ($141M), strategically fueling demand for its GPUs and expanding its AI ecosystem.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://www.ft.com/content/15eca6de-d4be-489d-baa6-765f25cdecf8, https://inflection.ai/inflection-ai-announces-1-3-billion-of-funding, https://www.bloomberg.com/news/articles/2023-06-08/ai-startup-cohere-raises-270-million-in-round-backed-by-oracle-nvidia, https://www.bloomberg.com/news/articles/2023-06-29/ai-video-startup-runway-raises-141-million-from-google-nvidia, https://decrypt.co/146757/ai-chatbot-startup-rockets-to-4-billion-valuation-with-microsoft-nvidia-backing</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.ft.com/content/15eca6de-d4be-489d-baa6-765f25cdecf8</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2023-01-10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Nvidia and Intel partner on AI computing efficiency</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Nvidia announced a collaboration with Intel around AI computing efficiency, a modest ecosystem development.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://blogs.nvidia.com/blog/2023/01/10/intel-partners-ai-computing-efficiency/</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://blogs.nvidia.com/blog/2023/01/10/intel-partners-ai-computing-efficiency/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2023-05-18</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Nvidia and ServiceNow partner on generative AI for IT service desks</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Nvidia-ServiceNow partnership applies generative AI to enterprise IT workflows, expanding enterprise AI use cases.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://www.investors.com/news/technology/nvda-stock-nvidia-servicenow-partnership-involves-generative-ai/</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.investors.com/news/technology/nvda-stock-nvidia-servicenow-partnership-involves-generative-ai/</t>
         </is>
       </c>
     </row>
@@ -7527,19 +8415,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>NVIDIA reports blowout Q1 FY24 data-center revenue and guidance</t>
+          <t>Nvidia fiscal Q1 earnings blowout forecast ignites $200B+ AI rally | Dell and Nvidia introduce Project Helix for on-premises generative AI</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>NVIDIA's blowout Q1 FY24 data-center revenue and guidance (event 2, 2022-05-24, one day before the inflection) is a high-impact earnings surprise that directly explains the strong BREAKOUT_UP on 2023-05-25. Source: https://nvidianews.nvidia.com/news/nvidia-announces-financial-results-for-first-quarter-fiscal-2024</t>
+          <t>The strongest breakout (sig=1.00) aligns with Nvidia's fiscal Q1 blowout forecast on 2023-05-24, which ignited a $200B+ AI-driven rally, per Reuters and Bloomberg (https://www.reuters.com/technology/nvidia-forecasts-second-quarter-revenue-above-estimates-2023-05-24/, https://www.bloomberg.com/news/articles/2023-05-24/nvidia-ignites-ai-related-stock-rally-after-blow-out-forecast). The Dell/Nvidia Project Helix announcement same day (https://nvidianews.nvidia.com/news/dell-technologies-and-nvidia-introduce-project-helix-for-secure-on-premises-generative-ai) is a minor contributor. High impact, one-day lag, and topical fit to a BREAKOUT_UP.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2023-02-23</t>
+          <t>2022-11-10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7548,26 +8436,26 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-19</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>OpenAI releases GPT-4 with multimodal capabilities</t>
+          <t>Nvidia introduces A800 GPU to circumvent U.S. China export restrictions | Nvidia bundles enterprise AI software with H100 systems at SC22</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>The GPT-4 release (event 1, 2023-03-14) is the nearest topically relevant event to the 2023-02-23 BREAKOUT_UP, but it occurs after the inflection with a sizable negative lag and only medium impact, so the causal link is weak. Source: https://openai.com/research/gpt-4</t>
+          <t>The 2022-11-10 breakout closely follows Nvidia's 2022-11-09 introduction of the A800 GPU to circumvent U.S. China export restrictions (high impact, one-day lag), per The Verge (https://www.theverge.com/2022/11/8/23447886/nvidia-a800-china-chip-ai-research-slowed-down-restrictions). Nvidia's SC22 H100 software bundling on 2022-11-14 (https://www.theregister.com/2022/11/14/nvidia_h100_software_bundle/) is a secondary product-driven catalyst within the window.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2022-11-10</t>
+          <t>2023-02-23</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -7576,19 +8464,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0.35</v>
+        <v>0.92</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>OpenAI launches ChatGPT, igniting generative-AI demand cycle</t>
+          <t>Nvidia fiscal Q4 earnings show growing lead in AI chip race | Nvidia CEO calls ChatGPT the 'iPhone moment of AI'</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>The ChatGPT launch (event 0, 2022-11-30) igniting the generative-AI demand cycle is topically aligned with a BREAKOUT_UP, but it occurs after the 2022-11-10 inflection, so the timing weakens the causal case. Source: https://openai.com/blog/chatgpt</t>
+          <t>This breakout exactly matches Nvidia's fiscal Q4 earnings on 2023-02-23 showing a growing lead in the AI chip race, with the stock up ~12% on the report, per CNBC and Reuters (https://www.cnbc.com/2023/02/23/nvidia-stock-up-12percent-on-earnings-ai-potential.html, https://www.reuters.com/technology/nvidia-results-show-its-growing-lead-ai-chip-race-2023-02-23/). The CEO's 'iPhone moment of AI' remark on 2023-02-13 (https://wccftech.com/nvidia-ceo-calls-chatgpt-as-one-of-the-greatest-thing-ever-done-for-computing-says-its-the-iphone-moment-of-ai/) added supporting momentum. Zero lag and high impact.</t>
         </is>
       </c>
     </row>

</xml_diff>